<commit_message>
alterações nas telas, logs e tabelas de utentes para o exercício Sit-and-Reach. Foram feitas melhorias na interface gráfica, correção de bugs e atualização dos dados dos utentes.
</commit_message>
<xml_diff>
--- a/tabelas_utentes/sit_and_reach_2_utentes.xlsx
+++ b/tabelas_utentes/sit_and_reach_2_utentes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I268"/>
+  <dimension ref="A1:I276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8458,15 +8458,11 @@
       </c>
     </row>
     <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
+      <c r="A268" t="n">
+        <v>21</v>
+      </c>
+      <c r="B268" t="n">
+        <v>165</v>
       </c>
       <c r="C268" t="inlineStr"/>
       <c r="D268" t="inlineStr">
@@ -8477,18 +8473,238 @@
       <c r="E268" t="n">
         <v>0</v>
       </c>
-      <c r="F268" t="inlineStr">
-        <is>
-          <t>5.79</t>
-        </is>
+      <c r="F268" t="n">
+        <v>5.79</v>
       </c>
       <c r="G268" t="n">
         <v>5.79</v>
       </c>
       <c r="H268" t="inlineStr"/>
-      <c r="I268" t="inlineStr">
-        <is>
-          <t>62</t>
+      <c r="I268" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>21</v>
+      </c>
+      <c r="B269" t="n">
+        <v>165</v>
+      </c>
+      <c r="C269" t="inlineStr"/>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>0</v>
+      </c>
+      <c r="F269" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="G269" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="H269" t="inlineStr"/>
+      <c r="I269" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>21</v>
+      </c>
+      <c r="B270" t="n">
+        <v>165</v>
+      </c>
+      <c r="C270" t="inlineStr"/>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>0</v>
+      </c>
+      <c r="F270" t="n">
+        <v>-3.83</v>
+      </c>
+      <c r="G270" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="H270" t="inlineStr"/>
+      <c r="I270" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>21</v>
+      </c>
+      <c r="B271" t="n">
+        <v>165</v>
+      </c>
+      <c r="C271" t="inlineStr"/>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>0</v>
+      </c>
+      <c r="F271" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="G271" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="H271" t="inlineStr"/>
+      <c r="I271" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>21</v>
+      </c>
+      <c r="B272" t="n">
+        <v>165</v>
+      </c>
+      <c r="C272" t="inlineStr"/>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>0</v>
+      </c>
+      <c r="F272" t="n">
+        <v>-7.33</v>
+      </c>
+      <c r="G272" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="H272" t="inlineStr"/>
+      <c r="I272" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>21</v>
+      </c>
+      <c r="B273" t="n">
+        <v>165</v>
+      </c>
+      <c r="C273" t="inlineStr"/>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>5</v>
+      </c>
+      <c r="F273" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="G273" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="H273" t="inlineStr"/>
+      <c r="I273" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>21</v>
+      </c>
+      <c r="B274" t="n">
+        <v>165</v>
+      </c>
+      <c r="C274" t="inlineStr"/>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>6</v>
+      </c>
+      <c r="F274" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="G274" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="H274" t="inlineStr"/>
+      <c r="I274" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>21</v>
+      </c>
+      <c r="B275" t="n">
+        <v>165</v>
+      </c>
+      <c r="C275" t="inlineStr"/>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>2</v>
+      </c>
+      <c r="F275" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="G275" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="H275" t="inlineStr"/>
+      <c r="I275" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr"/>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>5.65</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>165</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alterações de nome de janelas para "CAPACITA Project - Assessment Protocol", "CAPACITA Project - Assessment Complete" e "CAPACITA Project - Final Repetition Results". Alteração da ordem de exibição das telas de introdução. Adição de imagens.
</commit_message>
<xml_diff>
--- a/tabelas_utentes/sit_and_reach_2_utentes.xlsx
+++ b/tabelas_utentes/sit_and_reach_2_utentes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I276"/>
+  <dimension ref="A1:I280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8674,15 +8674,11 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
+      <c r="A276" t="n">
+        <v>21</v>
+      </c>
+      <c r="B276" t="n">
+        <v>165</v>
       </c>
       <c r="C276" t="inlineStr"/>
       <c r="D276" t="inlineStr">
@@ -8693,18 +8689,130 @@
       <c r="E276" t="n">
         <v>0.5</v>
       </c>
-      <c r="F276" t="inlineStr">
-        <is>
-          <t>5.65</t>
-        </is>
+      <c r="F276" t="n">
+        <v>5.65</v>
       </c>
       <c r="G276" t="n">
         <v>5.15</v>
       </c>
       <c r="H276" t="inlineStr"/>
-      <c r="I276" t="inlineStr">
+      <c r="I276" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>21</v>
+      </c>
+      <c r="B277" t="n">
+        <v>165</v>
+      </c>
+      <c r="C277" t="inlineStr"/>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>5</v>
+      </c>
+      <c r="F277" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="G277" t="n">
+        <v>0.4500000000000002</v>
+      </c>
+      <c r="H277" t="inlineStr"/>
+      <c r="I277" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>21</v>
+      </c>
+      <c r="B278" t="n">
+        <v>165</v>
+      </c>
+      <c r="C278" t="inlineStr"/>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>0</v>
+      </c>
+      <c r="F278" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G278" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H278" t="inlineStr"/>
+      <c r="I278" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>21</v>
+      </c>
+      <c r="B279" t="n">
+        <v>165</v>
+      </c>
+      <c r="C279" t="inlineStr"/>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="G279" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="H279" t="inlineStr"/>
+      <c r="I279" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
         <is>
           <t>165</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr"/>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>30</v>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>-43.53</t>
+        </is>
+      </c>
+      <c r="G280" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="H280" t="inlineStr"/>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>62</t>
         </is>
       </c>
     </row>

</xml_diff>